<commit_message>
ran significance tests and cleaned comments
</commit_message>
<xml_diff>
--- a/Analysis/Hybrid_Ablation/hybrid_ablation_friedman_tests.xlsx
+++ b/Analysis/Hybrid_Ablation/hybrid_ablation_friedman_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,16 @@
           <t>n_configs</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>p_holm</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>significant_holm</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,6 +489,12 @@
       <c r="G2" t="n">
         <v>3</v>
       </c>
+      <c r="H2" t="n">
+        <v>7.189751027225631e-18</v>
+      </c>
+      <c r="I2" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -506,6 +522,12 @@
       <c r="G3" t="n">
         <v>3</v>
       </c>
+      <c r="H3" t="n">
+        <v>3.96213819505597e-12</v>
+      </c>
+      <c r="I3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -533,6 +555,12 @@
       <c r="G4" t="n">
         <v>3</v>
       </c>
+      <c r="H4" t="n">
+        <v>4.847607949025935e-64</v>
+      </c>
+      <c r="I4" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -560,6 +588,12 @@
       <c r="G5" t="n">
         <v>3</v>
       </c>
+      <c r="H5" t="n">
+        <v>5.274615435877817e-20</v>
+      </c>
+      <c r="I5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -587,6 +621,12 @@
       <c r="G6" t="n">
         <v>3</v>
       </c>
+      <c r="H6" t="n">
+        <v>2.617591371228645e-14</v>
+      </c>
+      <c r="I6" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -614,6 +654,12 @@
       <c r="G7" t="n">
         <v>3</v>
       </c>
+      <c r="H7" t="n">
+        <v>4.46050625730004e-66</v>
+      </c>
+      <c r="I7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -641,6 +687,12 @@
       <c r="G8" t="n">
         <v>3</v>
       </c>
+      <c r="H8" t="n">
+        <v>1.523890173415963e-18</v>
+      </c>
+      <c r="I8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -668,6 +720,12 @@
       <c r="G9" t="n">
         <v>3</v>
       </c>
+      <c r="H9" t="n">
+        <v>4.05657205337039e-13</v>
+      </c>
+      <c r="I9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -694,6 +752,12 @@
       </c>
       <c r="G10" t="n">
         <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1.011816154762527e-61</v>
+      </c>
+      <c r="I10" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>